<commit_message>
tracking update 20.05.2026 17:12
</commit_message>
<xml_diff>
--- a/files/UAE_005_ФПЗ_ПРЕДВАРИТЕЛЬНЫЙ_17.05.2026.xlsx
+++ b/files/UAE_005_ФПЗ_ПРЕДВАРИТЕЛЬНЫЙ_17.05.2026.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D68F0E9-29AC-43AC-8DD3-9D10B24390D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EAF9AC3-4949-4BFD-B326-2B9A408E7F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ФПЗ_Э5" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="56">
   <si>
     <t xml:space="preserve">
 Артикул</t>
@@ -194,6 +194,18 @@
   </si>
   <si>
     <t>ИТОГО ФАКТ</t>
+  </si>
+  <si>
+    <t>MERCEDES-BENZ</t>
+  </si>
+  <si>
+    <t>A000989671013FBDW|Масло моторное|MERCEDES|229.52|5W-30|Синтетическое|Германия|3x5л</t>
+  </si>
+  <si>
+    <t>A000989681013FSEW|Масло моторное|MERCEDES|229.5|5W-40|Синтетическое|Германия|3x5л</t>
+  </si>
+  <si>
+    <t>A000989681011FSEW|Масло моторное|MERCEDES|229.5|5W-40|Синтетическое|Германия|12x1л</t>
   </si>
 </sst>
 </file>
@@ -886,7 +898,7 @@
   <cols>
     <col min="1" max="1" width="25.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="24.85546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="44.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.42578125" style="2" customWidth="1"/>
     <col min="4" max="4" width="11.7109375" style="3" customWidth="1"/>
     <col min="5" max="7" width="10.85546875" style="4" customWidth="1"/>
     <col min="8" max="8" width="10.42578125" style="5" customWidth="1"/>
@@ -2060,15 +2072,15 @@
         <v>633.95335130085243</v>
       </c>
       <c r="V2" s="31">
-        <v>800</v>
+        <v>820</v>
       </c>
       <c r="W2" s="32">
         <f>IFERROR((V2-U2)/U2,"")</f>
-        <v>0.26192250322271354</v>
+        <v>0.29347056580328135</v>
       </c>
       <c r="X2" s="33">
         <f t="shared" ref="X2:X9" si="7">V2*E2</f>
-        <v>9676800</v>
+        <v>9918720</v>
       </c>
       <c r="Y2" s="33">
         <f t="shared" ref="Y2:Y9" si="8">IFERROR(U2*E2,"")</f>
@@ -3072,15 +3084,15 @@
       <c r="AMG2" s="22"/>
       <c r="AMH2" s="22"/>
     </row>
-    <row r="3" spans="1:1022" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1022" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
         <v>46</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="D3" s="26">
         <v>5</v>
@@ -3145,15 +3157,15 @@
         <v>4213.336253299236</v>
       </c>
       <c r="V3" s="31">
-        <v>4850</v>
+        <v>4900</v>
       </c>
       <c r="W3" s="32">
         <f>IFERROR((V3-U3)/U3,"")</f>
-        <v>0.15110679718530109</v>
+        <v>0.1629738775686547</v>
       </c>
       <c r="X3" s="33">
         <f t="shared" si="7"/>
-        <v>2910000</v>
+        <v>2940000</v>
       </c>
       <c r="Y3" s="33">
         <f t="shared" si="8"/>
@@ -4162,10 +4174,10 @@
         <v>41</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D4" s="26">
         <v>5</v>
@@ -4202,7 +4214,7 @@
         <v>77.111971187641899</v>
       </c>
       <c r="O4" s="29">
-        <f t="shared" ref="O2:O8" si="15">K4*N4*1.0425</f>
+        <f t="shared" ref="O4:O8" si="15">K4*N4*1.0425</f>
         <v>2356.2451996270638</v>
       </c>
       <c r="P4" s="29">
@@ -4230,15 +4242,15 @@
         <v>3492.4552094546875</v>
       </c>
       <c r="V4" s="31">
-        <v>4780</v>
+        <v>4600</v>
       </c>
       <c r="W4" s="32">
         <f t="shared" ref="W4:W8" si="16">IFERROR((V4-U4)/U4,"")</f>
-        <v>0.36866465375409924</v>
+        <v>0.31712498060017918</v>
       </c>
       <c r="X4" s="33">
         <f t="shared" si="7"/>
-        <v>1147200</v>
+        <v>1104000</v>
       </c>
       <c r="Y4" s="33">
         <f t="shared" si="8"/>
@@ -5247,10 +5259,10 @@
         <v>42</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="D5" s="26">
         <v>1</v>
@@ -6396,15 +6408,15 @@
         <v>836.51496692659316</v>
       </c>
       <c r="V6" s="31">
-        <v>970</v>
+        <v>985</v>
       </c>
       <c r="W6" s="32">
         <f t="shared" si="16"/>
-        <v>0.1595727970819685</v>
+        <v>0.1775043351811742</v>
       </c>
       <c r="X6" s="33">
         <f t="shared" si="7"/>
-        <v>5028480</v>
+        <v>5106240</v>
       </c>
       <c r="Y6" s="33">
         <f t="shared" si="8"/>
@@ -6487,15 +6499,15 @@
         <v>1826.6838056618317</v>
       </c>
       <c r="V7" s="31">
-        <v>2950</v>
+        <v>3100</v>
       </c>
       <c r="W7" s="32">
         <f t="shared" si="16"/>
-        <v>0.61494835113577639</v>
+        <v>0.69706436899013791</v>
       </c>
       <c r="X7" s="33">
         <f t="shared" si="7"/>
-        <v>424800</v>
+        <v>446400</v>
       </c>
       <c r="Y7" s="33">
         <f t="shared" si="8"/>
@@ -6578,15 +6590,15 @@
         <v>527.90638782619988</v>
       </c>
       <c r="V8" s="31">
-        <v>785</v>
+        <v>840</v>
       </c>
       <c r="W8" s="32">
         <f t="shared" si="16"/>
-        <v>0.48700606414795239</v>
+        <v>0.59119120240035672</v>
       </c>
       <c r="X8" s="33">
         <f t="shared" si="7"/>
-        <v>113040</v>
+        <v>120960</v>
       </c>
       <c r="Y8" s="33">
         <f t="shared" si="8"/>
@@ -6714,7 +6726,7 @@
       <c r="W10" s="53"/>
       <c r="X10" s="63">
         <f>SUM(X2:X9)</f>
-        <v>22379040</v>
+        <v>22715040</v>
       </c>
       <c r="Y10" s="63">
         <f>SUM(Y2:Y9)</f>
@@ -6869,7 +6881,7 @@
       </c>
       <c r="Y14" s="65">
         <f>(X10-Y10)/Y10</f>
-        <v>0.23549230318067726</v>
+        <v>0.25404204498679173</v>
       </c>
     </row>
     <row r="15" spans="1:1022" ht="15.75" x14ac:dyDescent="0.25">

</xml_diff>